<commit_message>
Wave 13 deep pass: merge 56 verified brands from 42 under-covered sectors
81 fully verified (27 Yes / 29 Stretch / 25 No); NEW-W13 rows in consolidated
master and a W13 Deep Pass tab in the by-wave workbook.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TE8a9ptd2NGPUtY6iZfzkb
</commit_message>
<xml_diff>
--- a/reports/F1-New-Brands-By-Wave-2026-09.xlsx
+++ b/reports/F1-New-Brands-By-Wave-2026-09.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W7 Energy" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W8 Services &amp; Trading" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W9-12 Residues" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W13 Deep Pass" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'W1 Consumer'!$A$3:$M$69</definedName>
@@ -28,6 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'W7 Energy'!$A$3:$M$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'W8 Services &amp; Trading'!$A$3:$M$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'W9-12 Residues'!$A$3:$M$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'W13 Deep Pass'!$A$3:$M$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -110,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -128,6 +130,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -494,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -716,13 +724,28 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>W13 Deep Pass</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Wave 13 - Deep pass on the 42 under-covered sectors (21 Sep 2026): regional champions, family-owned, PE-owned; 81 fully verified, 56 kept</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
-        <v>286</v>
+      <c r="B23" s="3" t="n">
+        <v>342</v>
       </c>
     </row>
   </sheetData>
@@ -1887,6 +1910,3638 @@
     </row>
   </sheetData>
   <autoFilter ref="A3:M22"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Wave 13 - Deep pass on 42 under-covered sectors (regional champions, family-owned, PE-owned) - 56 brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>wave</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>sector_tab</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>priority_score</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>hq_country</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>niche</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>employees_est</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>size_band</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>tag</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>affordability</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>why_f1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>SaaS</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Info Edge (India)</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>infoedge.com</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Noida, India</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Online recruitment, real estate, and matrimony marketplace platforms (Naukri, Naukrigulf, 99acres, Jeevansathi)</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>5k-10k</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>5k-10k</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>INR 31.65B (~$381M at ~INR83/$) FY2025, up from INR 27.57B FY2024 (~15% YoY) - source: stockanalysis.com / company filings | INR 863.43B market cap (~$10.4B) as of Sept 2026 - source: companiesmarketcap.com | flags: Sector fit debatable: primarily an</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] India + Gulf 'precision matching' campaign timed to the region's F1 calendar (Abu Dhabi, Saudi Arabia, Qatar, Bahrain GPs), positioning Naukri/Naukrigulf as the platform connecting ambitious talent to global opportunity, into the s</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Photonics &amp; Optical</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Han's Laser Technology Industry Group Co., Ltd.</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>hanslaser.com</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Shenzhen, China</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Industrial laser processing/cutting/welding equipment and PCB equipment to thousands of manufacturing customers in consumer electronics, PCB, and AI/new-energy sectors globally</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>10k+ (~17,000-20,000, 2023-2025 company data)</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>~17,000-20,000, 2023-2025 company data</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>$2.67B / CNY18.7B, FY2025, +27% YoY, NPAT (excl. one-offs) +82% (Han's Laser investor release, reported via MarketScreener, 2026) | ~$15.3B market cap as of Sept 18, 2026 (PitchBook) | flags: Chinese tech exporter - general export-control/geopolitica</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Position Han's Laser as the precision-engineering backbone behind F1's manufacturing supply chain - 'the laser technology shaping the cars before they hit the track' - claiming the open photonics/laser-tech category, timed to its r</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Test &amp; Measurement</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Rohde &amp; Schwarz GmbH &amp; Co KG</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>rohde-schwarz.com</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>Munich, Germany</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>RF/microwave test equipment, broadcast, cybersecurity and secure communications, to a broad global customer base across telecom, defense, automotive and broadcast</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>10k+ (&gt;15,000 employees group-wide, ~10,000 in Germany, FY2024/25 company release)</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>&gt;15,000 employees group-wide, ~10,000 in Germany, FY2024/25 company release</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>€3.16B FY2024/25, +7.8% YoY, first time above €3B, record order backlog &gt;€5B (Rohde &amp; Schwarz press release, Nov 28, 2025) | Family-owned, no published valuation - passes on revenue alone per policy | flags: family-owned</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Anchor on R&amp;S's core competency in precision timing, RF and broadcast technology - the invisible infrastructure behind live sports broadcast and telemetry - positioning R&amp;S as the 'signal integrity' partner to F1's technology story</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>IoT &amp; Connectivity</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Ruijie Networks Co., Ltd.</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>ruijie.com</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>Fuzhou, China</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Enterprise networking and IoT connectivity equipment, sold in 140+ countries via 1,400+ Tier-2 partners, to enterprise, education, government and international customers</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>5k-10k (6,681-6,701 employees, 2025-2026, stockanalysis.com/Revelio Labs)</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>6,681-6,701 employees, 2025-2026, stockanalysis.com/Revelio Labs</t>
+        </is>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>RMB 14.32B (~$2.0B) FY2025, +22.37% YoY; overseas revenue growing even faster (+42-85% YoY across recent periods) (stockanalysis.com; BigGo Finance, 2026) | ~RMB 130.9B (~$18.4B) market cap as of Sept 18, 2026 (stockanalysis.com) | flags: internation</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Frame Ruijie as the AI-native networking backbone for global enterprise, leveraging its rapid international expansion (140+ countries) to use F1 as a platform for its overseas brand-building push, in the still-open enterprise-netwo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Machine Tools &amp; 3D Print</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>SCM Group S.p.A.</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>scmgroup.com</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>Rimini, Italy</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Woodworking and composite processing machinery</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k (cited range 1,000-5,000 employees; 26 locations worldwide)</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>cited range 1,000-5,000 employees; 26 locations worldwide</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>EUR900M consolidated group revenue, FY2024 (as of Dec 31, 2024), per SCM Group press release/RiminiToday (reported ~March 2025); parent SCM Group SpA standalone revenue EUR406.6M FY2024 with net profit EUR8.4M | n/a - family-owned, no published valua</t>
+        </is>
+      </c>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[VERIFIED NEW W13] Precision woodworking/composite-machinery technology story -- 'engineering the machines that shape performance materials' -- targeting the DACH/Italy manufacturing-technology seam, in a category not currently represented on the F1 </t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Machine Tools &amp; 3D Print</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Jyoti CNC Automation Limited</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>jyoti.co.in</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Rajkot, India</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>CNC machine tools (including simultaneous 5-axis machining centers)</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k (confirmed 3,845 employees as of Mar 2026, up 7.9% YoY, per company filings)</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>confirmed 3,845 employees as of Mar 2026, up 7.9% YoY, per company filings</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>FY2025 revenue ~INR2,191 crore / INR18.18B (~$249M est), up 35.8% YoY, per Screener.in/company financial filings | Market cap ~INR23,873 crore (~$2.85B) as of Sep 18, 2026, per stockanalysis.com/NSE -- clears the $1B bar | flags: recently listed (Jan</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] India's fastest-growing CNC machine-tool maker (35.8% YoY revenue growth, recent IPO) expanding into aerospace/EV/semiconductor machining -- a market-timing + 'engineering India's manufacturing rise' angle in an open category. | Al</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>DC Power &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Rittal GmbH &amp; Co. KG (Friedhelm Loh Group)</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>rittal.com</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>Herborn, Germany</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Enclosures, cooling and DC power infrastructure for data centers and industry</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>10k+ (Rittal alone cited at 12,000+; Friedhelm Loh Group ~15,000+ across 95+ international subsidiaries)</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>Rittal alone cited at 12,000+; Friedhelm Loh Group ~15,000+ across 95+ international subsidiaries</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>Friedhelm Loh Group revenue EUR3.1B (2024) growing to EUR3.2B (2025), per company reporting/Wikipedia -- growing YoY | n/a - family-owned, no published valuation (private) -- passes on revenue alone | flags: family-owned, no published valuation</t>
+        </is>
+      </c>
+      <c r="M10" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Data-center infrastructure boom angle -- Rittal's cooling/enclosure technology underpins the AI/data-center buildout, a live 'powering performance infrastructure' story that ties directly to F1's own technology-partner narrative, i</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Packaging &amp; Food Machinery</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Coesia Group</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>coesia.com</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Bologna, Italy</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Packaging and industrial process machinery (holding group of 21 companies)</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>5k-10k (8,000+ employees, per company materials)</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>8,000+ employees, per company materials</t>
+        </is>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>EUR2,107M (~$2.3B est), FY2024, per Coesia 2024 Sustainability Report/company reporting | n/a - family-owned (single shareholder), no published valuation -- passes on revenue alone | flags: family-owned, no published valuation; single-shareholder own</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Industrial-technology holding-group story -- Coesia's 21 companies engineer the precision machinery behind global packaging and manufacturing supply chains, an 'engineering behind the scenes' angle in an open category. | All hard f</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Packaging &amp; Food Machinery</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Marchesini Group S.p.A.</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>marchesini.com</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Bologna, Italy</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Pharmaceutical and packaging machinery</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k (1,612 employees, per company filings)</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>1,612 employees, per company filings</t>
+        </is>
+      </c>
+      <c r="K12" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>EUR369.4M FY2024, per company filings (aziende.it/Bilancio 2024); net result EUR62.7M -- strong margin | n/a - family-owned, no published valuation -- passes on revenue alone | flags: family-owned, no published valuation</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Precision pharma-machinery story -- Marchesini engineers the automated lines behind global medicine packaging, a 'precision at speed' angle resonant with F1 engineering culture, in an open category. | All hard filters pass: revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>TIC</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Applus Services, S.A. (Applus+)</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>applus.com</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>Barcelona, Spain</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Testing, inspection, certification (TIC) services across automotive, energy, industry and infrastructure sectors, 70+ countries</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>10k-10k+ (~26,000 employees, per company/TDR Capital materials, 2024)</t>
+        </is>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>~26,000 employees, per company/TDR Capital materials, 2024</t>
+        </is>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>9-month 2024 revenue EUR1.63B (+7.5% YoY, +7.6% organic); implies FY2024 ~EUR2.2-2.3B (source: Applus+ Q3 2024 Trading Update, applus.com) | Taken private June 2024 by TDR Capital + I Squared Capital for ~EUR1.7B deal value (source: TDR Capital, PE H</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Position Applus+ as F1's 'independent verification' story: the same rigor F1 uses to certify car legality, safety cells and parts maps onto Applus+'s testing/inspection/certification business - an open category with no incumbent TI</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Grid &amp; Transformers</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Elecnor, S.A.</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>elecnor.com</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>Madrid, Spain</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Electrical grid/transmission infrastructure EPC, energy, telecoms, water, rail and environmental project development across 50+ countries</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>10k+ (21,431 employees, per BME Exchange listing / 2024-2025 disclosures)</t>
+        </is>
+      </c>
+      <c r="J14" s="10" t="inlineStr">
+        <is>
+          <t>21,431 employees, per BME Exchange listing / 2024-2025 disclosures</t>
+        </is>
+      </c>
+      <c r="K14" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>EUR4.39B in FY2025 (+14.89% YoY vs EUR3.81B in FY2024) (source: MarketScreener 2025 Annual Results Report) | Market cap ~EUR3.25B (~$3.76-3.83B) as of May-June 2026 (source: stockanalysis.com/GuruFocus, 2026) | flags: est figures (input flag) - now s</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Grid modernization and electrification-of-everything narrative - Elecnor's transmission/grid EPC expertise pairs naturally with F1's push toward sustainable fuels, hybrid power units and race-weekend electrification (est). | All ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Materials &amp; Mech Parts</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>voestalpine AG</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>voestalpine.com</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>Linz, Austria</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Specialty steel, high-performance metals and materials technology for automotive, aerospace, rail, energy and industrial sectors</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>10k+ (~49,700 employees, FY2024/25, per voestalpine annual report)</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
+        <is>
+          <t>~49,700 employees, FY2024/25, per voestalpine annual report</t>
+        </is>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EUR15.7B in business year 2024/25 (source: voestalpine press release, June 2025) | Market cap ~$8.99B as of September 2026 (source: companiesmarketcap.com); clearly above the $1B bar under any recent measurement | flags: already a materials SUPPLIER </t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Turn an existing supplier relationship into a headline story: voestalpine already supplies precision components into F1 drivetrains via its Racing/HPM division - an official 'materials partner' deal would make that visible, credibl</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Automation &amp; Robotics</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Phoenix Contact GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>phoenixcontact.com</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>Blomberg, Germany</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Industrial connectivity, automation and electrification components sold in 100+ countries</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>10k+ (~22,000 employees group-wide, per company communications, 2022-2025)</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>~22,000 employees group-wide, per company communications, 2022-2025</t>
+        </is>
+      </c>
+      <c r="K16" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EUR3.04B in FY2024 (source: company disclosures cited via Zippia/craft.co, 2024); FY2024/2025 guidance from CEO Ulrich Leidecker anticipated revenue softening to ~EUR3.0B amid inventory de-stocking and geopolitical headwinds | n/a - family-owned, no </t>
+        </is>
+      </c>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Industrial IoT/connectivity-powers-performance narrative: Phoenix Contact's connectivity and automation components could be framed as the 'nervous system' technology behind trackside and factory data systems (est). | All hard filte</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Automation &amp; Robotics</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Weidmuller Group</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>weidmuller.com</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>Detmold, Germany</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Industrial connectivity and automation components</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>5k-10k (~5,500 employees group-wide, per company facts &amp; figures, 2024)</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="inlineStr">
+        <is>
+          <t>~5,500 employees group-wide, per company facts &amp; figures, 2024</t>
+        </is>
+      </c>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>EUR980M in 2024 (source: company disclosures, 2024) | n/a - family-owned, no published valuation; passes on revenue alone per family-owned exception | flags: est figures (input flag) - revenue confirmed at EUR980M vs the input's EUR1.1B estimate; dir</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Same industrial-connectivity-meets-precision-engineering story as larger peers, pitched at a scrappier/challenger-brand tier given its smaller-but-still-qualifying scale (est). | All hard filters pass: revenue EUR980M clears the $1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Packaging &amp; Food Machinery</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>GEA Group Aktiengesellschaft</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>gea.com</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>Duesseldorf, Germany</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Food and beverage processing machinery and process technology, global</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>10k+ (19,670 employees, per company disclosures)</t>
+        </is>
+      </c>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t>19,670 employees, per company disclosures</t>
+        </is>
+      </c>
+      <c r="K18" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>EUR5.5B in FY2025 (source: GEA 'reports profitable growth for 2025' press release, gea.com, 2026) | Market cap ~$10.4-12B as of 2026 (source: PitchBook/companiesmarketcap.com) | flags: input flag 'check dupe - may already be covered given scale' - no</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Precision process-engineering/technology-transfer narrative - GEA's food-tech engineering rigor and global-ambition scale mirror F1's own engineering-excellence story (est). | All hard filters pass: revenue EUR5.5B and market cap ~</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Packaging &amp; Food Machinery</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>SACMI Imola S.C.</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>sacmi.com</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>Imola, Italy</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Packaging, ceramics and beverage processing machinery, global</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k (4,756 employees at end of 2024, per SACMI Group 2024 results)</t>
+        </is>
+      </c>
+      <c r="J19" s="10" t="inlineStr">
+        <is>
+          <t>4,756 employees at end of 2024, per SACMI Group 2024 results</t>
+        </is>
+      </c>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>EUR1.728B in 2024, a record year (+12% per some coverage); net profit &gt;EUR200M, EBITDA &gt;EUR323M (source: SACMI Group 2024 results, sacmi.it, 2025) | n/a - cooperative-owned, no published valuation; passes on revenue alone under the family/cooperative</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Italian precision-engineering and 'record year' growth-momentum story, positioned alongside (or in place of) GEA Group in the Packaging &amp; Food Machinery slot given the two overlap (est). | All hard filters pass: revenue EUR1.728B c</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Grid &amp; Transformers</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Hitachi Energy India Limited</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>hitachienergy.com</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>Chennai, India</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Transformers, grid automation and HVDC equipment</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="K20" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>Annual revenue Rs.63.85B for FY ending Dec 2025 (~$768M USD, est FX conversion), +21.91% YoY (stockanalysis.com, 2026); Q1 FY27 (Jun 2026) revenue Rs.2,441 Cr | Market cap Rs.1,45,751.60 Cr (~$17.5B USD, est FX conversion) as of 18 Sep 2026, +54.5% o</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Lead with the HVDC/grid-modernization and energy-transition technology story, timed to F1's hybrid power-unit/sustainability narrative - grid/energy-infrastructure is an open sponsorship category on the current grid (est). | All ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Grid &amp; Transformers</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>GE Vernova T&amp;D India Limited</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>gevernova.com</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>Chennai, India</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Transformers, switchgear and grid equipment</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="K21" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>Rs.6,206.31 Cr FY2026 (~$746M USD, est FX conversion), +44.59% YoY; record order intake, EBITDA more than doubled, margins 27.2% (company FY25-26 results, 2026) | Market cap Rs.1,12,436.68 Cr (~$13.5B USD, est FX conversion) as of 21 Sep 2026 (NSE li</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Energy-transition and grid-reliability technology story - GE Vernova's 'electrify and decarbonize' positioning pairs with F1's sustainability push, and the grid-equipment sponsor category is currently unclaimed on the grid (est). |</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Materials &amp; Mech Parts</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>The Timken Company</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>timken.com</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>North Canton, Ohio, USA</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Bearings and mechanical power transmission products</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="J22" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="K22" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L22" s="7" t="inlineStr">
+        <is>
+          <t>$4.6B in FY2025, +0.2% YoY (Timken Q4/FY2025 results press release, 4 Feb 2026) - far exceeds the $100M hard bar | Market cap ~$9.61B USD as of Jul 2026 (stockanalysis.com) - far exceeds the $1B hard bar | flags: Revenue growth essentially flat (+0.2</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Precision-engineering/performance-under-extreme-load story - bearings and power-transmission components are a natural technical fit for F1's engineering narrative, and the category is open on the current grid (est). | All hard filt</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>OT &amp; Physical Security</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Brinks Company</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>brinks.com</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>Richmond, Virginia, US</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Cash logistics, ATM services and secure valuables transport to thousands of bank and retail customers globally</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>10k+ (~20,000-21,000, est)</t>
+        </is>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
+        <is>
+          <t>~20,000-21,000, est</t>
+        </is>
+      </c>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>$5.26B FY2025, +4.97% YoY (confirmed via WebSearch, Brink's Q4/FY2025 results release, reported ~Feb 2026) | Market cap ~$4.4-4.5B as of Sep 17, 2026 (confirmed via WebSearch, stockanalysis.com/companiesmarketcap.com)</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Global secure-logistics/fintech-infrastructure story - 'trusted at speed' - open category, timed to Brink's tech-driven cash-management modernization push. | All hard filters pass cleanly: revenue and valuation well above bars, pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Trading &amp; Crypto</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>XTB S.A.</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>xtb.com</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>Warsaw, Poland</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Retail CFD/forex brokerage and trading platform, pan-European reach</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="J24" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="K24" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L24" s="7" t="inlineStr">
+        <is>
+          <t>PLN 2.12B / ~$570M FY2025 (+14.3% YoY); TTM ~$833M as of Sept 2026 (stockanalysis.com) | Market cap ~$4.9B as of early Sept 2026 (stockanalysis.com) | flags: compliance-frame: leveraged retail CFD trading faces gambling-adjacent advertising/regulator</t>
+        </is>
+      </c>
+      <c r="M24" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] 'Return to the grid' angle - XTB already has a 2010 McLaren precedent; reintroduce as a modern trading-technology partner in an open CFD/retail-investing category, leaning on real-time data/precision parallels with F1. | All hard f</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Travel &amp; Hospitality</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Barcelo Hotel Group</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>barcelo.com</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>Palma de Mallorca, Spain</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Multinational hotel group (Royal Hideaway, Occidental brands), Spain, Caribbean, Americas, Europe, Africa</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="J25" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="K25" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L25" s="7" t="inlineStr">
+        <is>
+          <t>Barceló Group turnover &gt;€7.5B FY2024 (+~12-16% YoY vs €6.7B in 2023), €661M EBITDA, €301.8M net profit, debt eliminated (dominicantoday.com / Barceló Group 2024 Annual Report) | Private, no published valuation; family-owned, passes on revenue alone p</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Global-hospitality-scale angle - a debt-free, family-run multinational hotel group spanning the Americas, Europe and Africa, offering F1 an open hospitality-category partner untouched by existing grid sponsors. | All hard filters p</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>56 Robotics AI</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>84</v>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Delta Electronics</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>deltaww.com</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>Taipei, Taiwan</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Industrial automation and robotics (robot arms, machine vision) plus power electronics</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="J26" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="K26" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L26" s="7" t="inlineStr">
+        <is>
+          <t>$14B+ group revenue, FY2024 (public results) | ~$30B+ market cap (Taiwan Stock Exchange, public) | flags: robotics is only one of several segments -- power electronics, EV components and ICT infrastructure make up most of group revenue</t>
+        </is>
+      </c>
+      <c r="M26" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] "Invisible engineering" angle: Delta's power electronics and robotics as the precision technology powering both EV drivetrains and the pit garage -- a supplier story for an unclaimed robotics/automation category. | All hard filters</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>32 Defense &amp; Industrial AI</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>84</v>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Diehl Stiftung &amp; Co. KG (Diehl Group)</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>diehl.com</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>Nuremberg, Germany</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Precision-guided munitions and air-defense systems (Diehl Defence), plus industrial/metering technology</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="J27" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="K27" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
+          <t>€4,695.8M (2024, +20.9% YoY, per Diehl Group annual report) | No published valuation (family-owned) -- passes on revenue alone per the family-owned exemption | flags: family-owned with limited public financial disclosure beyond headline figures; defe</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Precision-under-pressure engineering story: Diehl's guided-systems and aerospace-grade manufacturing tolerances as a natural technology-partner narrative for F1's own precision-engineering culture, told through its commercial (non-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>IoT &amp; Connectivity</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="n">
+        <v>84</v>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Nordic Semiconductor ASA</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>nordicsemi.com</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>Trondheim, Norway</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Low-power wireless (Bluetooth LE, cellular IoT) chips and modules</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="J28" s="10" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="K28" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L28" s="7" t="inlineStr">
+        <is>
+          <t>Q2 2025 revenue $164M, +28-33% YoY (investing.com); FY2025 run-rate est. ~$600M+ | $2.59B (Q2 2025) rising to ~$4B (June 2026) market cap (Oslo: NOD) | flags: search did not confirm or rule out a minority stake by a Norwegian state fund (e.g., Folket</t>
+        </is>
+      </c>
+      <c r="M28" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] "Connectivity at the edge" story: Nordic's ultra-low-power wireless chips as the invisible nervous system analogy for F1's trackside and in-car telemetry sensor networks -- an open IoT-silicon category on the grid. | All hard filte</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Commercial Vehicles</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="n">
+        <v>84</v>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>Bucher Industries AG</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>bucherindustries.com</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>Niederweningen, Switzerland</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Municipal vehicles (street sweepers, Bucher Municipal), agricultural machinery (Kuhn) and specialty vehicle equipment</t>
+        </is>
+      </c>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="K29" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>CHF 2.9B (~$3.68B USD) in FY2025, reported with 2026 annual results (companiesmarketcap.com/investing.com, Mar 2026) - far exceeds the $100M hard bar | Market cap ranged ~CHF 2.88B-$4.9B across 2026 reporting dates (disfold.com/companiesmarketcap.com</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[VERIFIED NEW W13] Precision-agriculture technology story via the Kuhn brand (data-driven farming, efficiency/performance) paired with Bucher's global-champion narrative as a Swiss engineering group - commercial/municipal vehicles is an open sponsor </t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Staffing &amp; Talent</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>84</v>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Gi Group Holding S.p.A.</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>gigroup.com</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>Milan, Italy</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Staffing, HR services and workforce solutions across 37+ countries</t>
+        </is>
+      </c>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="K30" s="10" t="inlineStr">
+        <is>
+          <t>verified-new</t>
+        </is>
+      </c>
+      <c r="L30" s="7" t="inlineStr">
+        <is>
+          <t>€4.7B / ~$4.9B FY2024, up 22.7% YoY (Il Sole 24 Ore / Gi Group Holding 2024 Annual Report, reported 2025) | Private, no published valuation; founder-owned, passes on revenue alone per policy | flags: founder/family-owned, no published valuation; head</t>
+        </is>
+      </c>
+      <c r="M30" s="7" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Open category on the 2026 grid - position as the workforce/talent partner behind the pit crews, engineers and global operations teams that keep an F1 team running, tying into Gi Group's 37-country reach and growth story. | All hard</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Devtools &amp; Integration</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Cockroach Labs</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>cockroachlabs.com</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>New York, NY, USA</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>Distributed SQL database (CockroachDB) for enterprise developers/infrastructure teams</t>
+        </is>
+      </c>
+      <c r="I31" s="11" t="inlineStr">
+        <is>
+          <t>201-1k</t>
+        </is>
+      </c>
+      <c r="J31" s="11" t="inlineStr">
+        <is>
+          <t>201-1k</t>
+        </is>
+      </c>
+      <c r="K31" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L31" s="9" t="inlineStr">
+        <is>
+          <t>$145.8M FY2024 (company-disclosed); ARR reported to have tripled YoY heading into 2025 - source: Contrary Research / Cockroach Labs press materials | $5B post-money, Dec 2021 Series F - source: PitchBook/Crunchbase; no updated public valuation disclo</t>
+        </is>
+      </c>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Position CockroachDB as the always-on, zero-downtime data infrastructure behind split-second telemetry and strategy decisions, into the still-open enterprise database/infra sponsorship slot. | All hard filters pass (revenue $145.8M</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>13 AI Agents</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Ada Support</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>ada.cx</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>Toronto, Canada</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>Agentic AI customer-service platform for enterprise support teams</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr">
+        <is>
+          <t>201-1k</t>
+        </is>
+      </c>
+      <c r="J32" s="11" t="inlineStr">
+        <is>
+          <t>201-1k</t>
+        </is>
+      </c>
+      <c r="K32" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L32" s="9" t="inlineStr">
+        <is>
+          <t>~$70.6M ARR (2024, third-party est., getlatka.com); company reports &gt;100% YoY ARR growth in FY ending ~Mar 2026 (Ada press release/BusinessWire, Mar 2026) -- implies ARR now well above $50M and growing &gt;50% YoY (est) | $1.2B (Series C, 2021, reaffirm</t>
+        </is>
+      </c>
+      <c r="M32" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[VERIFIED NEW W13] "Always-on precision" story: agentic AI that never misses a customer call, echoing pit-wall decision speed -- first mover into an unclaimed AI customer-service category on the grid. | Hard filters appear to pass (ARR growing 100%+ </t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>Electronic Parts</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>AT&amp;S Austria Technologie &amp; Systemtechnik AG</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>ats.net</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>Leoben, Austria</t>
+        </is>
+      </c>
+      <c r="H33" s="9" t="inlineStr">
+        <is>
+          <t>Printed circuit boards and IC substrates to mobile devices, automotive, industrial and medical customers globally, including AI/data-center substrate demand</t>
+        </is>
+      </c>
+      <c r="I33" s="11" t="inlineStr">
+        <is>
+          <t>10k+ (~14,000 est.)</t>
+        </is>
+      </c>
+      <c r="J33" s="11" t="inlineStr">
+        <is>
+          <t>~14,000 est.</t>
+        </is>
+      </c>
+      <c r="K33" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L33" s="9" t="inlineStr">
+        <is>
+          <t>€1.7-1.8B FY2025/26 with a 23% EBITDA margin, driven by AI/data-center substrate demand (AT&amp;S investor release, 2026) | ~€5.95B (~$6.4B) market cap, early Sept 2026 (companiesmarketcap.com) | flags: customer concentration: Apple is ~20-25% of the Mob</t>
+        </is>
+      </c>
+      <c r="M33" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Lead with AT&amp;S's AI/data-center substrate growth story - positioning it as the precision-substrate technology enabling next-gen high-performance computing, tying into F1's own compute/AI-driven engineering narrative, in the open PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>Machine Tools &amp; 3D Print</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>Fair Friend Group (FFG)</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>ffg-tw.com</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>Taipei, Taiwan</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>Machine tools (CNC lathes/mills, multiple brands including Feeler, Victor, MAG) via ~94 companies/50 factories in 10 countries</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>10k+ (est ~13,000; group scale of 94 companies/50 factories across 10 countries is consistent with 10k+, but not independently itemized in an official filing)</t>
+        </is>
+      </c>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>est ~13,000; group scale of 94 companies/50 factories across 10 countries is consistent with 10k+, but not independently itemized in an official filing</t>
+        </is>
+      </c>
+      <c r="K34" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L34" s="9" t="inlineStr">
+        <is>
+          <t>Estimates vary and are not tightly dated: ~$1.4B (ZoomInfo, dated ~May 2026) vs ~$3.3B group-wide turnover (FFG corporate materials, undated) vs ~$1.8B machine-tool-division-only (CENS, 2014). All comfortably clear the &gt;$100M hard bar regardless of w</t>
+        </is>
+      </c>
+      <c r="M34" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Global manufacturing-technology story: FFG is described as the world's #3 machine-tool group supplying precision equipment to automotive/aerospace primes across 10 countries -- an 'engineering the machines behind performance' angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>Automation &amp; Robotics</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>Hans Turck GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>turck.com</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>Muelheim an der Ruhr, Germany</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>Industrial sensors and connectivity products for factory automation</t>
+        </is>
+      </c>
+      <c r="I35" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k (est ~4,600; company-published figures conflict, ranging from ~2,510 (2021) to ~5,000 across data aggregators - none current or official)</t>
+        </is>
+      </c>
+      <c r="J35" s="11" t="inlineStr">
+        <is>
+          <t>2021) to ~5,000 across data aggregators - none current or official</t>
+        </is>
+      </c>
+      <c r="K35" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L35" s="9" t="inlineStr">
+        <is>
+          <t>Uncertain/conflicting: most recent confirmed official figure is EUR470.3M (2021); third-party aggregators show a very wide and unreliable range (some as low as $50-100M, clearly inconsistent with the company's own 2019-2021 disclosures of EUR600-640M</t>
+        </is>
+      </c>
+      <c r="M35" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Sensor/connectivity precision-engineering narrative in the same vein as Phoenix Contact/Weidmuller, best pursued once current financials are confirmed directly with the company (est). | Likely clears all hard filters (revenue almos</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>Automation &amp; Robotics</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>Pilz GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>pilz.com</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>Ostfildern, Germany</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="inlineStr">
+        <is>
+          <t>Safety automation systems for industrial machinery</t>
+        </is>
+      </c>
+      <c r="I36" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k (2,504 employees worldwide as of Dec 31, 2024, +1.1% YoY, per Pilz 2024 annual press release)</t>
+        </is>
+      </c>
+      <c r="J36" s="11" t="inlineStr">
+        <is>
+          <t>2,504 employees worldwide as of Dec 31, 2024, +1.1% YoY, per Pilz 2024 annual press release</t>
+        </is>
+      </c>
+      <c r="K36" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L36" s="9" t="inlineStr">
+        <is>
+          <t>EUR341M in 2024, down 21% YoY after three very good prior years - weak, particularly in Germany/Europe; export share rose to 79% (source: Pilz 2024 financial-year press release) | n/a - family-owned, no published valuation; passes on revenue alone pe</t>
+        </is>
+      </c>
+      <c r="M36" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Safety-culture/engineering-excellence narrative tying Pilz's industrial safety-automation expertise to F1's own uncompromising approach to driver and crew safety - best timed for when the company's order book recovers (est). | Reve</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>Construction &amp; Field Svc</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>SafetyCulture Pty Ltd</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>safetyculture.com</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>Sydney, Australia</t>
+        </is>
+      </c>
+      <c r="H37" s="9" t="inlineStr">
+        <is>
+          <t>Field inspection, safety and workflow software (iAuditor/SafetyCulture platform) used across construction, industrial and field operations</t>
+        </is>
+      </c>
+      <c r="I37" s="11" t="inlineStr">
+        <is>
+          <t>201-1k (~910 employees as of mid-2026, per CB Insights/company data)</t>
+        </is>
+      </c>
+      <c r="J37" s="11" t="inlineStr">
+        <is>
+          <t>~910 employees as of mid-2026, per CB Insights/company data</t>
+        </is>
+      </c>
+      <c r="K37" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L37" s="9" t="inlineStr">
+        <is>
+          <t>Conflicting third-party estimates: ~$90.3M ARR (2025, per one aggregator) vs. ~$197.6M total revenue (2025, per another); an earlier confirmed data point showed $84.4M revenue in FY2023 (+32% YoY). No official company-disclosed figure found in this p</t>
+        </is>
+      </c>
+      <c r="M37" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Safety-technology narrative: SafetyCulture's inspection/safety-workflow software mirrors F1's rigorous approach to pit-crew, marshal and paddock safety - a natural 'safety innovation partner' story once current financials are confi</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Commercial Vehicles</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>Zoomlion Heavy Industry Science and Technology Co., Ltd.</t>
+        </is>
+      </c>
+      <c r="F38" s="11" t="inlineStr">
+        <is>
+          <t>zoomlion.com</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
+        <is>
+          <t>Changsha, China</t>
+        </is>
+      </c>
+      <c r="H38" s="9" t="inlineStr">
+        <is>
+          <t>Construction machinery, cranes and heavy equipment</t>
+        </is>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="K38" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L38" s="9" t="inlineStr">
+        <is>
+          <t>RMB 52.107B in FY2025 (~$7.2B USD, est FX conversion), +14.58% YoY; net profit RMB 4.858B, +38.01% YoY (Zoomlion 2025 results, PR Newswire, 2 Apr 2026) - far exceeds the $100M hard bar | Market cap (est) in the multi-billion-dollar range for this dua</t>
+        </is>
+      </c>
+      <c r="M38" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Global-expansion and heavy-engineering performance story - Zoomlion's rapid international growth (59% of revenue, manufacturing across 8+ countries) pairs with F1's global-market growth narrative; heavy machinery/construction is an</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>Commercial Vehicles</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>Krone Commercial Vehicle Group</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>krone-cv.com</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>Werlte, Germany</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>Truck trailers and semi-trailers to thousands of logistics and trucking fleets, mainly in Europe</t>
+        </is>
+      </c>
+      <c r="I39" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k (~4,500, est; not independently reconfirmed)</t>
+        </is>
+      </c>
+      <c r="J39" s="11" t="inlineStr">
+        <is>
+          <t>~4,500, est; not independently reconfirmed</t>
+        </is>
+      </c>
+      <c r="K39" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L39" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Group turnover ~€2.3B (FY2024/25) / ~€2.4B ($2.6B) FY2024, down from €3.2B prior year (confirmed via WebSearch, krone-trailer.com press release &amp; Commercial Motor, Feb 2026) | Private, no published valuation (family-owned; passes hard bar on revenue </t>
+        </is>
+      </c>
+      <c r="M39" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Open commercial-logistics/trailer-manufacturing category; European trade/logistics visibility angle timed to Krone's demand-recovery narrative. | All hard filters pass (still profitable per company statement, headcount/audience/own</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>OT &amp; Physical Security</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>Eulen S.A.</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>eulen.com</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>Madrid, Spain</t>
+        </is>
+      </c>
+      <c r="H40" s="9" t="inlineStr">
+        <is>
+          <t>Facility management and security services (incl. converged physical/cyber security) to thousands of client contracts across 11 countries, mainly Spain/LatAm</t>
+        </is>
+      </c>
+      <c r="I40" s="11" t="inlineStr">
+        <is>
+          <t>10k+ (~73,000-82,000, confirmed via WebSearch, Sep 2026)</t>
+        </is>
+      </c>
+      <c r="J40" s="11" t="inlineStr">
+        <is>
+          <t>~73,000-82,000, confirmed via WebSearch, Sep 2026</t>
+        </is>
+      </c>
+      <c r="K40" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L40" s="9" t="inlineStr">
+        <is>
+          <t>~€1.79B (~$1.9-2B) consolidated sales, FY2024 (confirmed via WebSearch, Sep 2026) | Private, no published valuation (family-owned; passes hard bar on revenue per brief rule) | flags: family-owned, no published valuation; historically thin net margins</t>
+        </is>
+      </c>
+      <c r="M40" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Iberian/LatAm growth story leveraging Eulen's converged security/tech (SOC, IP surveillance) positioning; open category; best pursued once the succession dispute resolves. | Hard filters technically pass (revenue clears the family-</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>Staffing &amp; Talent</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>Outsourcing Inc.</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>outsourcing.co.jp</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>Tokyo, Japan</t>
+        </is>
+      </c>
+      <c r="H41" s="9" t="inlineStr">
+        <is>
+          <t>Staffing, engineering and business-process outsourcing services, Japan and internationally</t>
+        </is>
+      </c>
+      <c r="I41" s="11" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="J41" s="11" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="K41" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L41" s="9" t="inlineStr">
+        <is>
+          <t>JPY 749.6B / ~$4.99B FY2023 (+8.6% YoY; staffingindustry.com, reported Feb 2024) - most recent figure independently confirmed in search; FY2024/25 results not verified | Market cap ~¥221bn (~$1.4-1.5B) per a 2026-dated Stockopedia pull, though the un</t>
+        </is>
+      </c>
+      <c r="M41" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Precision-engineering and global-workforce-logistics story - Outsourcing Inc. keeps aviation, automotive and manufacturing lines staffed worldwide, a natural tie-in to F1's own high-precision, globally-mobile operations. | Hard fil</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>Travel &amp; Hospitality</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>Hotelbeds Group (HBX Group)</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="inlineStr">
+        <is>
+          <t>hotelbeds.com</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr">
+        <is>
+          <t>Palma de Mallorca, Spain</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>B2B hotel-bed bank / travel wholesaler serving 60,000+ travel-trade distributors globally</t>
+        </is>
+      </c>
+      <c r="I42" s="11" t="inlineStr">
+        <is>
+          <t>5k-10k</t>
+        </is>
+      </c>
+      <c r="J42" s="11" t="inlineStr">
+        <is>
+          <t>5k-10k</t>
+        </is>
+      </c>
+      <c r="K42" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L42" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">€693M with €363M core profit, FY2024 (Reuters/dominicantoday-sourced coverage of Barceló... [Hotelbeds figures per company reporting, 2025) | Post-IPO market cap ~€2.84-2.93B / ~$2.9-3.0B as of Feb 2025 listing (Reuters/MarketScreener/TradingView) | </t>
+        </is>
+      </c>
+      <c r="M42" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Global travel-logistics story - position Hotelbeds/HBX as the infrastructure behind the travel trade that gets fans, teams and hospitality guests to Grand Prix weekends worldwide. | Hard filters pass (revenue and post-IPO market ca</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>17 AI Cloud &amp; Data</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>Iris Energy (IREN)</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>irisenergy.co</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>Sydney, Australia</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>AI/GPU cloud infrastructure and data centers (pivoted from bitcoin mining)</t>
+        </is>
+      </c>
+      <c r="I43" s="11" t="inlineStr">
+        <is>
+          <t>201-1k</t>
+        </is>
+      </c>
+      <c r="J43" s="11" t="inlineStr">
+        <is>
+          <t>201-1k</t>
+        </is>
+      </c>
+      <c r="K43" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L43" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$501M FY2025 (macrotrends/stockanalysis); AI Cloud ARR surpassed $500M annualized by early 2026 (company blog/press) | ~$14-18B market cap (NASDAQ, Sept 2026, stockanalysis.com/CNN) | flags: heavy single-customer concentration: Microsoft is expected </t>
+        </is>
+      </c>
+      <c r="M43" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] "Engine behind the AI era" story: IREN's data-center/power-engineering precision (renewable-powered AI compute at scale) paired against F1 teams' own AI/compute-hungry strategy operations. | Hard bars pass comfortably (revenue, val</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>32 Defense &amp; Industrial AI</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>Poongsan Corporation</t>
+        </is>
+      </c>
+      <c r="F44" s="11" t="inlineStr">
+        <is>
+          <t>poongsan.co.kr</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>Seoul, South Korea</t>
+        </is>
+      </c>
+      <c r="H44" s="9" t="inlineStr">
+        <is>
+          <t>Ammunition/defense systems and copper alloy materials</t>
+        </is>
+      </c>
+      <c r="I44" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="J44" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="K44" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L44" s="9" t="inlineStr">
+        <is>
+          <t>$3.68B trailing 12 months (mid-2026, stockanalysis.com) | ~$1.54B market cap (Korea Exchange, Sept 2026, PitchBook/MarketScreener) | flags: National Pension Service (a state pension fund) holds ~11.4% -- a minority state-linked stake; ammunition/defe</t>
+        </is>
+      </c>
+      <c r="M44" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Precision-engineering-under-pressure story: position Poongsan's defense-grade metallurgy and copper-alloy engineering as an 'the margins matter' technology-supplier narrative, distinct from ammunition messaging. | Hard filters pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>Electronic Parts</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>Walsin Lihwa Corporation</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>walsin.com</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>Taipei, Taiwan</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>Wire and cable, stainless steel and electronic materials to industrial, construction, utility and manufacturing customers across Asia, the US and Europe</t>
+        </is>
+      </c>
+      <c r="I45" s="11" t="inlineStr">
+        <is>
+          <t>5k-10k (7,651 employees, company/GlobalData data, 2025-2026)</t>
+        </is>
+      </c>
+      <c r="J45" s="11" t="inlineStr">
+        <is>
+          <t>7,651 employees, company/GlobalData data, 2025-2026</t>
+        </is>
+      </c>
+      <c r="K45" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L45" s="9" t="inlineStr">
+        <is>
+          <t>NT$174.24B (~$5.6B) FY2025, down -2.83% YoY; 9-month 2025 net sales NT$132.38B (stockanalysis.com; Walsin Lihwa investor release, 2026) | ~NT$143.58B (~$4.6B) market cap, Sept 2026 (stockanalysis.com) | flags: thin and volatile margins - gross margin</t>
+        </is>
+      </c>
+      <c r="M45" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Position Walsin Lihwa around the materials science behind next-gen EV charging and grid infrastructure (its wire &amp; cable and electronic-materials lines) - an infrastructure-of-the-future angle distinct from typical high-tech F1 spo</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>Machine Tools &amp; 3D Print</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>Ace Micromatic Group</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>acemicromatic.net</t>
+        </is>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="inlineStr">
+        <is>
+          <t>CNC machine tools</t>
+        </is>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k (est; group-wide figure uncertain -- flagship Ace Designers Ltd confirmed at ~1,600-1,700 employees, but multi-entity group total not independently verified; input estimate ~4,000)</t>
+        </is>
+      </c>
+      <c r="J46" s="11" t="inlineStr">
+        <is>
+          <t>est; group-wide figure uncertain -- flagship Ace Designers Ltd confirmed at ~1,600-1,700 employees, but multi-entity group total not independently verified; input estimate ~4,000</t>
+        </is>
+      </c>
+      <c r="K46" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L46" s="9" t="inlineStr">
+        <is>
+          <t>Confirmed only at the flagship-entity level: Ace Designers Ltd revenue ~INR2,240 crore (~$269M est) for FY ended Mar 2024, per company filings/Tofler. Group-wide consolidated revenue could not be independently confirmed; the group has publicly target</t>
+        </is>
+      </c>
+      <c r="M46" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] India's largest machine-tool group riding the 'Make in India' manufacturing-growth story -- an angle built on India's industrial rise, pending firmer confirmation of export reach and consolidated financials. | Hard filters technica</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr">
+        <is>
+          <t>Materials &amp; Mech Parts</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>fischerwerke GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t>fischer.group</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>Waldachtal, Germany</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>Fixing systems and fasteners (construction, DIY, automotive)</t>
+        </is>
+      </c>
+      <c r="I47" s="11" t="inlineStr">
+        <is>
+          <t>5k-10k (confirmed ~5,900 employees, 2023, up ~300 YoY)</t>
+        </is>
+      </c>
+      <c r="J47" s="11" t="inlineStr">
+        <is>
+          <t>confirmed ~5,900 employees, 2023, up ~300 YoY</t>
+        </is>
+      </c>
+      <c r="K47" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L47" s="9" t="inlineStr">
+        <is>
+          <t>EUR1.16B group turnover, FY2023 (reported Feb 2024) -- a company record, up 2% YoY; no independently confirmed 2024/2025 total-group figure found in this search pass (est for currency; separately, its Automotive division alone was projected at ~EUR20</t>
+        </is>
+      </c>
+      <c r="M47" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] German engineering-heritage story (75+ years, record 2023 turnover) -- a 'precision fixing technology' angle tying fischer's fastening/engineering innovation to F1 performance-engineering themes, in an open category. | Hard filters</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>Grid &amp; Transformers</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>Siemens Energy India Limited</t>
+        </is>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>siemensenergy.com</t>
+        </is>
+      </c>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>Mumbai, India</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="inlineStr">
+        <is>
+          <t>Transformers, switchgear and grid equipment for power generation, transmission and renewable integration</t>
+        </is>
+      </c>
+      <c r="I48" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="J48" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="K48" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L48" s="9" t="inlineStr">
+        <is>
+          <t>Revenue ~Rs.9,436 Cr (~$1.1B USD, est FX conversion) per FY figures cited via Screener.in/INDmoney (2026); Q4 FY26 quarterly revenue Rs.2,394 Cr | Market cap Rs.1,13,214 Cr (~$13.6B USD, est FX conversion) as of 11 Sep 2026 (INDmoney) | flags: Brand-</t>
+        </is>
+      </c>
+      <c r="M48" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Position explicitly as 'Siemens Energy' (distinct from Siemens AG) and lead with the energy-transition/grid-modernization story, timed to a team's sustainability or power-unit announcement, while proactively clarifying the entity s</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>OT &amp; Physical Security</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>Sohgo Security Services Co., Ltd. (ALSOK)</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>alsok.co.jp</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>Tokyo, Japan</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="inlineStr">
+        <is>
+          <t>Guarding, alarm monitoring and cash transport security services to thousands of corporate and individual clients, ~15% Japan market share</t>
+        </is>
+      </c>
+      <c r="I49" s="11" t="inlineStr">
+        <is>
+          <t>10k+ (~40,000, est)</t>
+        </is>
+      </c>
+      <c r="J49" s="11" t="inlineStr">
+        <is>
+          <t>~40,000, est</t>
+        </is>
+      </c>
+      <c r="K49" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L49" s="9" t="inlineStr">
+        <is>
+          <t>Consolidated net sales &gt;¥520B (~$3.96B) for FY ended March 2025 (confirmed via WebSearch, financial data aggregators, Sep 2026) | Market cap ~$3.62B as of Aug 24, 2026 (confirmed via WebSearch) | flags: predominantly domestic-Japan revenue base despi</t>
+        </is>
+      </c>
+      <c r="M49" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Anchor to the Japanese Grand Prix (Suzuka) as home-market activation; security-tech/monitoring innovation story, timed to the 2025 ALSOK rebrand seeking greater global visibility. | Hard filters pass (revenue, valuation, headcount,</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>Travel &amp; Hospitality</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>EIH Limited (Oberoi Hotels)</t>
+        </is>
+      </c>
+      <c r="F50" s="11" t="inlineStr">
+        <is>
+          <t>oberoihotels.com</t>
+        </is>
+      </c>
+      <c r="G50" s="11" t="inlineStr">
+        <is>
+          <t>New Delhi, India</t>
+        </is>
+      </c>
+      <c r="H50" s="9" t="inlineStr">
+        <is>
+          <t>Ultra-luxury hospitality under the Oberoi and Trident hotel brands, ~30 properties across India, Egypt, Mauritius, Indonesia and Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="I50" s="11" t="inlineStr">
+        <is>
+          <t>5k-10k (est) - EIH Limited reported ~5,708 employees per recent aggregator data (2025/2026); note source figures conflict across trackers, treat as uncertain (est)</t>
+        </is>
+      </c>
+      <c r="J50" s="11" t="inlineStr">
+        <is>
+          <t>est</t>
+        </is>
+      </c>
+      <c r="K50" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L50" s="9" t="inlineStr">
+        <is>
+          <t>~$310-335M USD (est conversion) - consolidated revenue of INR 2,743.15 crore in FY25 (year ended Mar 2025), +9.23% YoY; Q4 FY25 PAT grew 6% YoY to INR 263 crore, confirming profitability (source: Business Standard, May 2025; screener.in FY25 filings)</t>
+        </is>
+      </c>
+      <c r="M50" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Position Oberoi/Trident as F1's first dedicated ultra-luxury hospitality partner - VIP paddock-adjacent stays and bespoke travel packages for teams/sponsors/high-net-worth fans around Middle East and Asia-Pacific race weekends, lev</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>09 Fintech</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>Stone Co</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>stone.co</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>Sao Paulo, Brazil</t>
+        </is>
+      </c>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>Payments, digital banking, and software platform for Brazilian merchants (SMBs)</t>
+        </is>
+      </c>
+      <c r="I51" s="11" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="J51" s="11" t="inlineStr">
+        <is>
+          <t>10k+</t>
+        </is>
+      </c>
+      <c r="K51" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L51" s="9" t="inlineStr">
+        <is>
+          <t>R$13.4B (2025), +16% YoY, ~$2.5B USD equiv. - source: SEC Form 20-F/6-K filings, stockanalysis.com | $3.91B market cap (2026) - source: stockanalysis.com | flags: Single-market (Brazil-only) concentration is a real reservation on global-brand fit des</t>
+        </is>
+      </c>
+      <c r="M51" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] A Sao Paulo Grand Prix (Interlagos)-timed activation showcasing Stone's payments infrastructure as 'the engine behind Brazilian commerce', framed as a stepping stone toward the company's stated future international expansion. | All</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>09 Fintech</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>Globe Fintech Innovations (GCash / Mynt)</t>
+        </is>
+      </c>
+      <c r="F52" s="11" t="inlineStr">
+        <is>
+          <t>gcash.com</t>
+        </is>
+      </c>
+      <c r="G52" s="11" t="inlineStr">
+        <is>
+          <t>Manila, Philippines</t>
+        </is>
+      </c>
+      <c r="H52" s="9" t="inlineStr">
+        <is>
+          <t>Mobile wallet, digital payments, and financial services super-app for Philippine consumers/merchants</t>
+        </is>
+      </c>
+      <c r="I52" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="J52" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="K52" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L52" s="9" t="inlineStr">
+        <is>
+          <t>Highly variable estimates: ~$1.4B (Oct 2025 est.) vs. other estimates of $100-200M/yr; Globe's equity-earnings share from Mynt grew 64% YoY (PHP3.8B to PHP6.1B) in 2025 - sources: Caproasia, Bloomberg (Aug 2025), insiderph.com - figure genuinely unce</t>
+        </is>
+      </c>
+      <c r="M52" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] A Southeast Asia financial-inclusion growth story timed to the Singapore Grand Prix's regional reach, positioning GCash as the super-app powering millions of underbanked consumers, into an open digital-wallet sponsorship slot. | Ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="inlineStr">
+        <is>
+          <t>09 Fintech</t>
+        </is>
+      </c>
+      <c r="D53" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E53" s="11" t="inlineStr">
+        <is>
+          <t>Fawry</t>
+        </is>
+      </c>
+      <c r="F53" s="11" t="inlineStr">
+        <is>
+          <t>fawry.com</t>
+        </is>
+      </c>
+      <c r="G53" s="11" t="inlineStr">
+        <is>
+          <t>Cairo, Egypt</t>
+        </is>
+      </c>
+      <c r="H53" s="9" t="inlineStr">
+        <is>
+          <t>Digital payments and e-finance platform for Egyptian consumers and merchants</t>
+        </is>
+      </c>
+      <c r="I53" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="J53" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k</t>
+        </is>
+      </c>
+      <c r="K53" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L53" s="9" t="inlineStr">
+        <is>
+          <t>EGP 8.65B (2025), +57% YoY (from EGP 5.51B) ~ $175-180M USD equiv. - source: stockanalysis.com/company filings | EGP 66.26B market cap as of Sept 2026 (~$1.3-1.4B USD at ~EGP48-50/USD); note the market cap was as low as EGP 49.74B (~$1.0B) as recentl</t>
+        </is>
+      </c>
+      <c r="M53" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] A MENA digital-payments growth story timed to the region's F1 races (Bahrain, Saudi Arabia, Qatar, Abu Dhabi GPs), positioning Fawry as the infrastructure behind Egypt's cashless-economy shift, into an open MENA fintech sponsorship</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>Commercial Vehicles</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>TAFE (Tractors and Farm Equipment Limited)</t>
+        </is>
+      </c>
+      <c r="F54" s="11" t="inlineStr">
+        <is>
+          <t>tafe.com</t>
+        </is>
+      </c>
+      <c r="G54" s="11" t="inlineStr">
+        <is>
+          <t>Chennai, India</t>
+        </is>
+      </c>
+      <c r="H54" s="9" t="inlineStr">
+        <is>
+          <t>Tractors and farm equipment (Massey Ferguson India license, Eicher tractors) to hundreds of thousands of Indian and export-market farmers</t>
+        </is>
+      </c>
+      <c r="I54" s="11" t="inlineStr">
+        <is>
+          <t>5k-10k (~10,000, est; not independently reconfirmed)</t>
+        </is>
+      </c>
+      <c r="J54" s="11" t="inlineStr">
+        <is>
+          <t>~10,000, est; not independently reconfirmed</t>
+        </is>
+      </c>
+      <c r="K54" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L54" s="9" t="inlineStr">
+        <is>
+          <t>~$1.6B / INR 16,000+ crore annual turnover, current/general figure not broken out by fiscal year (confirmed via WebSearch of TAFE corporate profile, Sep 2026) | Private, no published valuation (family-owned; passes hard bar on revenue per brief rule)</t>
+        </is>
+      </c>
+      <c r="M54" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Open 'agriculture/heavy machinery' category; tie to TAFE's global-expansion push (Africa/Asia export growth) and precision-engineering story rather than the mass-farmer buyer base. | All hard filters pass (revenue, family-owned no-</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="inlineStr">
+        <is>
+          <t>Gulf Sovereign &amp; Tourism</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>Dubai Investments PJSC</t>
+        </is>
+      </c>
+      <c r="F55" s="11" t="inlineStr">
+        <is>
+          <t>dubaiinvestments.com</t>
+        </is>
+      </c>
+      <c r="G55" s="11" t="inlineStr">
+        <is>
+          <t>Dubai, UAE</t>
+        </is>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>Diversified investment holding - real estate, industrial manufacturing, financial investments - across Gulf subsidiaries</t>
+        </is>
+      </c>
+      <c r="I55" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k (~5,000, est, across subsidiaries)</t>
+        </is>
+      </c>
+      <c r="J55" s="11" t="inlineStr">
+        <is>
+          <t>~5,000, est, across subsidiaries</t>
+        </is>
+      </c>
+      <c r="K55" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L55" s="9" t="inlineStr">
+        <is>
+          <t>~$729M annual revenue as of Feb 2026 reporting; AED 1.5B net profit in 2025 (confirmed via WebSearch, Sep 2026) | ~AED 7B / $1.9B market cap, DFM-listed (est, not independently reconfirmed with a current 2026 figure) | flags: diversified holding stru</t>
+        </is>
+      </c>
+      <c r="M55" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Industrial/real-estate diversification story tied to UAE's non-oil private-investment growth narrative; open 'diversified holding' category, though brand focus would need sharpening. | Hard filters pass (revenue, valuation, headcou</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>Gulf Sovereign &amp; Tourism</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>Jabal Omar Development Company</t>
+        </is>
+      </c>
+      <c r="F56" s="11" t="inlineStr">
+        <is>
+          <t>jabalomar.com.sa</t>
+        </is>
+      </c>
+      <c r="G56" s="11" t="inlineStr">
+        <is>
+          <t>Mecca, Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="H56" s="9" t="inlineStr">
+        <is>
+          <t>Hospitality and real estate development adjacent to the Grand Mosque (hotel towers, retail) serving the global pilgrim/tourist market</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
+          <t>1k-5k (~1,500, est)</t>
+        </is>
+      </c>
+      <c r="J56" s="11" t="inlineStr">
+        <is>
+          <t>~1,500, est</t>
+        </is>
+      </c>
+      <c r="K56" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L56" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAR 2.11B (~$560M) FY2025, +11.17% YoY; net profit surged to SAR 2.39B (from SAR 200M in 2024) (confirmed via WebSearch, Argaam/stockanalysis.com, Sep 2026) | ~SAR 16.7B / $4.46B market cap as of March 2026 (confirmed via search, carried from input) </t>
+        </is>
+      </c>
+      <c r="M56" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] Tie to Jabal Omar's explosive 2025 profit growth and Saudi Vision 2030 tourism/sports diversification narrative; open 'hospitality/pilgrimage tourism development' category. | Hard filters pass on available evidence (revenue, valuat</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C57" s="11" t="inlineStr">
+        <is>
+          <t>Gulf Sovereign &amp; Tourism</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E57" s="11" t="inlineStr">
+        <is>
+          <t>Lulu Retail Holdings PLC</t>
+        </is>
+      </c>
+      <c r="F57" s="11" t="inlineStr">
+        <is>
+          <t>luluretail.com</t>
+        </is>
+      </c>
+      <c r="G57" s="11" t="inlineStr">
+        <is>
+          <t>Abu Dhabi, UAE</t>
+        </is>
+      </c>
+      <c r="H57" s="9" t="inlineStr">
+        <is>
+          <t>Hypermarkets and retail (GCC's largest grocery/retail chain, also a tourist shopping destination) to tens of millions of shoppers</t>
+        </is>
+      </c>
+      <c r="I57" s="11" t="inlineStr">
+        <is>
+          <t>10k+ (53,459 employees, Lulu Group International, as of June 2026, confirmed via WebSearch)</t>
+        </is>
+      </c>
+      <c r="J57" s="11" t="inlineStr">
+        <is>
+          <t>53,459 employees, Lulu Group International, as of June 2026, confirmed via WebSearch</t>
+        </is>
+      </c>
+      <c r="K57" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L57" s="9" t="inlineStr">
+        <is>
+          <t>H1 2025 revenue $4.1B, +5.9% YoY; net income $127M, +9.1% YoY (confirmed via WebSearch, luluretail.com H1 2025 results); full-year ~$8.3B (est, consistent with input) | ~$6.5B market cap, ADX-listed post Nov-2024 IPO (est, carried from input, not ind</t>
+        </is>
+      </c>
+      <c r="M57" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] GCC's largest hypermarket chain as a consumer-facing regional retail sponsor, tied to Abu Dhabi GP home-market activation and the recent landmark IPO growth story; open grocery/retail category. | Hard filters pass (revenue, valuati</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>Staffing &amp; Talent</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>Kanzhun Limited (Boss Zhipin)</t>
+        </is>
+      </c>
+      <c r="F58" s="11" t="inlineStr">
+        <is>
+          <t>ir.kanzhun.com</t>
+        </is>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>Beijing, China</t>
+        </is>
+      </c>
+      <c r="H58" s="9" t="inlineStr">
+        <is>
+          <t>Online recruitment platform (Boss Zhipin) connecting job seekers and employers</t>
+        </is>
+      </c>
+      <c r="I58" s="11" t="inlineStr">
+        <is>
+          <t>5k-10k</t>
+        </is>
+      </c>
+      <c r="J58" s="11" t="inlineStr">
+        <is>
+          <t>5k-10k</t>
+        </is>
+      </c>
+      <c r="K58" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L58" s="9" t="inlineStr">
+        <is>
+          <t>RMB 7,355.7M / $1,007.7M FY2024 (Kanzhun IR/Nasdaq press release, March 2025); RMB 8,267.5M / $1,182.2M FY2025 | Market cap ~$6-7B through 2025, $7.14B as of Aug 2026 (stockanalysis.com/Yahoo Finance) | flags: revenue and user base overwhelmingly Chi</t>
+        </is>
+      </c>
+      <c r="M58" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[VERIFIED NEW W13] China/APAC market-entry story for F1 - use Kanzhun's AI-driven hiring technology and stated push into new geographies (Vietnam, Argentina, Brazil) as the hook for an emerging-market or technology-partner angle. | Hard filters pass </t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C59" s="11" t="inlineStr">
+        <is>
+          <t>Trading &amp; Crypto</t>
+        </is>
+      </c>
+      <c r="D59" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E59" s="11" t="inlineStr">
+        <is>
+          <t>CoinDCX</t>
+        </is>
+      </c>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>coindcx.com</t>
+        </is>
+      </c>
+      <c r="G59" s="11" t="inlineStr">
+        <is>
+          <t>Mumbai, India</t>
+        </is>
+      </c>
+      <c r="H59" s="9" t="inlineStr">
+        <is>
+          <t>Cryptocurrency exchange and trading platform, India and UAE/MENA (via BitOasis acquisition)</t>
+        </is>
+      </c>
+      <c r="I59" s="11" t="inlineStr">
+        <is>
+          <t>201-1k</t>
+        </is>
+      </c>
+      <c r="J59" s="11" t="inlineStr">
+        <is>
+          <t>201-1k</t>
+        </is>
+      </c>
+      <c r="K59" s="11" t="inlineStr">
+        <is>
+          <t>verified-stretch</t>
+        </is>
+      </c>
+      <c r="L59" s="9" t="inlineStr">
+        <is>
+          <t>~$141M ARR as of June 2025 (getlatka.com); YoY growth rate not independently confirmed | $2.45B post-money, Oct 15, 2025 (Coinbase minority investment; TradingView/Coinbase blog) | flags: revenue figure is ARR, not confirmed audited FY/TTM revenue; g</t>
+        </is>
+      </c>
+      <c r="M59" s="9" t="inlineStr">
+        <is>
+          <t>[VERIFIED NEW W13] India/MENA growth-market story - CoinDCX as the exchange of record for the world's fastest-growing crypto user base, offering F1 a foothold distinct from the Western crypto sponsors already on the grid. | Valuation and capacity-to-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:M59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>